<commit_message>
V7.9 r6: R9 building 3D, pipe/duct ports, logic completion, English UI, EPMS tenant billing
- 3D page runs the R9 office/architecture layer (r9office.js) with a LIVE adapter;
  AHU/OAU/tower/exptank/bypass Blender models rebuilt with real nozzles/collars
- r9_connections.py: 117 pipe/duct ends meet the model ports (CI step)
- v79_r6.py: AHU-01/02 OA/RA, OAU cascade, TEF, kitchen KEF/MAU, relief,
  B1 plant-room ventilation, corridor sensors, floor CHW requests to the plant,
  expansion CHW setpoint/kW, coil/isolation instruments, EPMS billing data
- Tenant billing page/Px + EPMS export register; SOO and EPMS docs
- All web pages, 3D page and register in English; site name removed
- Tests: 30/30 layer tests PASS

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AewrLSrp3pc2fo4Kic8Aj3
</commit_message>
<xml_diff>
--- a/registers/ALT_V79_Equipment_Register.xlsx
+++ b/registers/ALT_V79_Equipment_Register.xlsx
@@ -461,7 +461,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ทะเบียนอุปกรณ์ ALT_CP_Ref_V7_9</t>
+          <t>ALT_CP_Ref_V7_9 equipment register</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -469,12 +469,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ใช้ทำอะไร</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ไฟล์เดียวที่บอกว่าไซต์นี้มีอุปกรณ์อะไรบ้าง builder อ่านไฟล์นี้แล้วสร้าง station, Field IO, point mapping, 3D และแบบ 2D ให้ตรงกัน</t>
+          <t>The single file that says which equipment the site has. The builder reads it and generates the station, Field IO, point mapping, 3D and 2D drawings consistently.</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>chiller / CHP / CDP / CT อย่างละ 6 slot (01-02 = เครื่องเดิมของ V7.8, 03-06 = slot ขยาย) · Installed = Y/N</t>
+          <t>chiller / CHP / CDP / CT, 6 slots each (01-02 = existing V7.8 units, 03-06 = expansion slots) · Installed = Y/N</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sensor เพิ่มเติม (SNS01...) ใส่กี่แถวก็ได้ อย่างน้อย 6 slot · Kind: Temp, RH, Pressure, DP, Flow, Power, Level, Generic</t>
+          <t>additional sensors (SNS01...), any number of rows, at least 6 slots · Kind: Temp, RH, Pressure, DP, Flow, Power, Level, Generic</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>AHU ประจำชั้น 2-8 (ชั้น 1 = AHU01/02, OAU01, FCU01-04 ของ V7.8) · Installed = Y/N</t>
+          <t>floor AHUs 2-8 (floor 1 = AHU01/02, OAU01 of V7.8) · Installed = Y/N</t>
         </is>
       </c>
     </row>
@@ -522,43 +522,43 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ระบบในอนาคต (fire alarm, fire protection, lighting, power) · ใส่อุปกรณ์ทีละแถว: ชั้น, ตำแหน่ง X/Y/Z (มม.), Point ใน station → ขึ้นใน 3D เป็นจุดพร้อมสถานะ</t>
+          <t>future systems (fire alarm, fire protection, lighting, power) · one device per row: floor, X/Y/Z position (mm), station point -&gt; shown in 3D with its status</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>เพิ่มอุปกรณ์ (วิธีที่ 1, ไม่ต้องสร้างใหม่)</t>
+          <t>Add equipment (method 1, no rebuild)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ใน Workbench ตั้ง &lt;slot&gt;_Installed = true (เช่น CH03_Installed) → logic นับเครื่องนั้นทันที → ต่อ Field IO กลุ่ม &lt;slot&gt; → ทดสอบ P2P</t>
+          <t>In Workbench set &lt;slot&gt;_Installed = true (e.g. CH03_Installed) -&gt; the logic counts the unit at once -&gt; wire the Field IO group &lt;slot&gt; -&gt; P2P test</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>เพิ่มอุปกรณ์ (วิธีที่ 2, สร้างใหม่)</t>
+          <t>Add equipment (method 2, rebuild)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>แก้ไฟล์นี้ (Installed = Y, Protocol, Device) → สั่ง make_v79.py --register ไฟล์นี้ → ได้ config.bog + ทะเบียนจุด + 3D ใหม่ที่ตรงกัน</t>
+          <t>Edit this file (Installed = Y, Protocol, Device) -&gt; run make_v79.py --register &lt;this file&gt; -&gt; new config.bog + point register + 3D that match</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ลดอุปกรณ์</t>
+          <t>Remove equipment</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ตั้ง Installed = N (หรือ &lt;slot&gt;_Installed = false ใน Workbench) → เครื่องนั้นไม่ถูกเลือก ไม่ถูกสั่งเดิน และเป็นเงาจางใน 3D</t>
+          <t>Set Installed = N (or &lt;slot&gt;_Installed = false in Workbench) -&gt; the unit is not selected, never started and shown as a ghost in 3D</t>
         </is>
       </c>
     </row>

</xml_diff>